<commit_message>
Migrate the 4 Visiting International child pages (section-interior)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-section-interior.report.xlsx
+++ b/tools/importer/reports/import-section-interior.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="266">
   <si>
     <t>_reportFile</t>
   </si>
@@ -151,7 +151,7 @@
     <t>nav</t>
   </si>
   <si>
-    <t>2026-10-07T16:47:57.765Z</t>
+    <t>2026-10-07T18:44:48.172Z</t>
   </si>
   <si>
     <t>rc.report.json</t>
@@ -750,6 +750,63 @@
   </si>
   <si>
     <t>https://lsa.umich.edu/lsa/prospective-students/undergraduate/what-are-the-liberal-arts-.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/academics.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/academics</t>
+  </si>
+  <si>
+    <t>2026-10-07T19:32:16.787Z</t>
+  </si>
+  <si>
+    <t>Academics | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international/visiting-international/academics.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/admissions-and-requirements.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/admissions-and-requirements</t>
+  </si>
+  <si>
+    <t>2026-10-07T19:32:14.782Z</t>
+  </si>
+  <si>
+    <t>Admissions and Requirements | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international/visiting-international/admissions-and-requirements.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/admitted-students.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/admitted-students</t>
+  </si>
+  <si>
+    <t>2026-10-07T19:32:22.618Z</t>
+  </si>
+  <si>
+    <t>Admitted Students | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international/visiting-international/admitted-students.html</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/student-life.report.json</t>
+  </si>
+  <si>
+    <t>lsa/prospective-students/international/visiting-international/student-life</t>
+  </si>
+  <si>
+    <t>2026-10-07T19:32:19.854Z</t>
+  </si>
+  <si>
+    <t>https://lsa.umich.edu/lsa/prospective-students/international/visiting-international/student-life.html</t>
   </si>
   <si>
     <t>lsa/prospective-students/undergraduate/admissions/undergraduate-application.report.json</t>
@@ -1153,7 +1210,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="50" customWidth="1"/>
@@ -2774,6 +2831,146 @@
         <v>246</v>
       </c>
     </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>247</v>
+      </c>
+      <c r="B47" t="s">
+        <v>143</v>
+      </c>
+      <c r="C47" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" t="s">
+        <v>13</v>
+      </c>
+      <c r="E47" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" t="s">
+        <v>248</v>
+      </c>
+      <c r="G47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H47" t="s">
+        <v>102</v>
+      </c>
+      <c r="I47" t="s">
+        <v>249</v>
+      </c>
+      <c r="J47" t="s">
+        <v>250</v>
+      </c>
+      <c r="K47" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>252</v>
+      </c>
+      <c r="B48" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" t="s">
+        <v>13</v>
+      </c>
+      <c r="D48" t="s">
+        <v>13</v>
+      </c>
+      <c r="E48" t="s">
+        <v>13</v>
+      </c>
+      <c r="F48" t="s">
+        <v>253</v>
+      </c>
+      <c r="G48" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" t="s">
+        <v>102</v>
+      </c>
+      <c r="I48" t="s">
+        <v>254</v>
+      </c>
+      <c r="J48" t="s">
+        <v>255</v>
+      </c>
+      <c r="K48" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>257</v>
+      </c>
+      <c r="B49" t="s">
+        <v>12</v>
+      </c>
+      <c r="C49" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" t="s">
+        <v>13</v>
+      </c>
+      <c r="F49" t="s">
+        <v>258</v>
+      </c>
+      <c r="G49" t="s">
+        <v>15</v>
+      </c>
+      <c r="H49" t="s">
+        <v>102</v>
+      </c>
+      <c r="I49" t="s">
+        <v>259</v>
+      </c>
+      <c r="J49" t="s">
+        <v>235</v>
+      </c>
+      <c r="K49" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>261</v>
+      </c>
+      <c r="B50" t="s">
+        <v>12</v>
+      </c>
+      <c r="C50" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" t="s">
+        <v>13</v>
+      </c>
+      <c r="E50" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" t="s">
+        <v>262</v>
+      </c>
+      <c r="G50" t="s">
+        <v>15</v>
+      </c>
+      <c r="H50" t="s">
+        <v>102</v>
+      </c>
+      <c r="I50" t="s">
+        <v>263</v>
+      </c>
+      <c r="J50" t="s">
+        <v>264</v>
+      </c>
+      <c r="K50" t="s">
+        <v>265</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>